<commit_message>
Add Q10436 Windows Playwright reproduction
</commit_message>
<xml_diff>
--- a/artifacts/任务规格转化.xlsx
+++ b/artifacts/任务规格转化.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格转化" sheetId="1" r:id="R87f67043d9834b4c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格转化" sheetId="1" r:id="Raebc36aeefc54092"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -378,7 +378,7 @@
         <x:v>核心操作链</x:v>
       </x:c>
       <x:c r="B9" s="5" t="str">
-        <x:v>读取场景与字幕；配置Chromium；创建浏览器上下文；操作字幕与倍速；发送键盘事件；检查可访问属性；整理报告</x:v>
+        <x:v>读取场景与字幕；配置Chromium；隔离浏览器状态；操作字幕与倍速；发送键盘事件；检查可访问属性；整理报告</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="48" customHeight="1">
@@ -423,10 +423,10 @@
     </x:row>
     <x:row r="15" ht="33" customHeight="1">
       <x:c r="A15" s="5" t="str">
-        <x:v>业务核对点</x:v>
+        <x:v>可验证点</x:v>
       </x:c>
       <x:c r="B15" s="5" t="str">
-        <x:v>回环服务、上下文隔离、字幕选中、倍速记忆、键盘状态、ARIA属性、报告主键和输入保全</x:v>
+        <x:v>回环服务、状态隔离、字幕选中、倍速记忆、键盘状态、ARIA属性、报告主键和输入保全</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="33" customHeight="1">

</xml_diff>